<commit_message>
Add outputs from the data-prep using the library-index.xlsx as input data
</commit_message>
<xml_diff>
--- a/examples/library-index.xlsx
+++ b/examples/library-index.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc350584/Documents/github/jcudlc-generate-index/example-input-data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jc350584/Documents/github/jcudlc/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F59C9753-57BD-FC4E-9209-A979B6FCB11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD47CA3A-47D6-1544-BDA2-12318BDA98A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25880" yWindow="1140" windowWidth="24040" windowHeight="18300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" r:id="rId1"/>
@@ -735,12 +735,6 @@
   </cellStyleXfs>
   <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -847,6 +841,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1064,979 +1064,979 @@
   <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="16.1640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="45.33203125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="24.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="5" customWidth="1"/>
-    <col min="6" max="6" width="15.1640625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="28" style="5" customWidth="1"/>
-    <col min="8" max="8" width="40.1640625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="15.1640625" style="5" customWidth="1"/>
-    <col min="10" max="10" width="33.83203125" style="5" customWidth="1"/>
-    <col min="11" max="11" width="14.6640625" style="5" customWidth="1"/>
-    <col min="12" max="12" width="11.83203125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="98.1640625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="21.5" style="5" customWidth="1"/>
-    <col min="15" max="15" width="16.6640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="28.1640625" style="5" customWidth="1"/>
-    <col min="17" max="17" width="32.33203125" style="5" customWidth="1"/>
-    <col min="18" max="16384" width="8.83203125" style="5"/>
+    <col min="1" max="1" width="16.1640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="45.33203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="24.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="15.1640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="28" style="3" customWidth="1"/>
+    <col min="8" max="8" width="40.1640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15.1640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="33.83203125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="98.1640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="21.5" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="28.1640625" style="3" customWidth="1"/>
+    <col min="17" max="17" width="32.33203125" style="3" customWidth="1"/>
+    <col min="18" max="16384" width="8.83203125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="4"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="2"/>
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="I4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="K4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="L4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="M4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="N4" s="7" t="s">
+      <c r="N4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="P4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="Q4" s="8" t="s">
+      <c r="Q4" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="L5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="M5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="N5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="O5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="Q5" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="M6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="N6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="O6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="P6" s="10" t="s">
+      <c r="P6" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="Q6" s="11" t="s">
+      <c r="Q6" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="H7" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="J7" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="M7" s="13" t="s">
+      <c r="M7" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="N7" s="13" t="s">
+      <c r="N7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="O7" s="13" t="s">
+      <c r="O7" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="P7" s="13" t="s">
+      <c r="P7" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="14" t="s">
+      <c r="Q7" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="J8" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13" t="s">
+      <c r="K8" s="11"/>
+      <c r="L8" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="M8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="N8" s="13" t="s">
+      <c r="N8" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="O8" s="13" t="s">
+      <c r="O8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="P8" s="13" t="s">
+      <c r="P8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="Q8" s="14" t="s">
+      <c r="Q8" s="12" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="J9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13" t="s">
+      <c r="K9" s="11"/>
+      <c r="L9" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="M9" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="N9" s="13" t="s">
+      <c r="N9" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="O9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="P9" s="13" t="s">
+      <c r="P9" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="14" t="s">
+      <c r="Q9" s="12" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="15" customHeight="1">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13" t="s">
+      <c r="K10" s="11"/>
+      <c r="L10" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="M10" s="13" t="s">
+      <c r="M10" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="N10" s="13" t="s">
+      <c r="N10" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="O10" s="13" t="s">
+      <c r="O10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="P10" s="13" t="s">
+      <c r="P10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="Q10" s="14" t="s">
+      <c r="Q10" s="12" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="G11" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="I11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="J11" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16" t="s">
+      <c r="K11" s="14"/>
+      <c r="L11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="M11" s="16" t="s">
+      <c r="M11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="N11" s="16" t="s">
+      <c r="N11" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="O11" s="16" t="s">
+      <c r="O11" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="P11" s="16" t="s">
+      <c r="P11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Q11" s="17" t="s">
+      <c r="Q11" s="15" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19" t="s">
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19" t="s">
+      <c r="G12" s="17"/>
+      <c r="H12" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="I12" s="19" t="s">
+      <c r="I12" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19" t="s">
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="19" t="s">
+      <c r="M12" s="17"/>
+      <c r="N12" s="17"/>
+      <c r="O12" s="17"/>
+      <c r="P12" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="Q12" s="20" t="s">
+      <c r="Q12" s="18" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="22" t="s">
+      <c r="B13" s="20"/>
+      <c r="C13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22" t="s">
+      <c r="D13" s="20"/>
+      <c r="E13" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22" t="s">
+      <c r="F13" s="20"/>
+      <c r="G13" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22" t="s">
+      <c r="H13" s="20"/>
+      <c r="I13" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22" t="s">
+      <c r="K13" s="20"/>
+      <c r="L13" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22" t="s">
+      <c r="M13" s="20"/>
+      <c r="N13" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="O13" s="22"/>
-      <c r="P13" s="22" t="s">
+      <c r="O13" s="20"/>
+      <c r="P13" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="Q13" s="23" t="s">
+      <c r="Q13" s="21" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22" t="s">
+      <c r="C14" s="20"/>
+      <c r="D14" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22" t="s">
+      <c r="E14" s="20"/>
+      <c r="F14" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22" t="s">
+      <c r="G14" s="20"/>
+      <c r="H14" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22" t="s">
+      <c r="I14" s="20"/>
+      <c r="J14" s="20"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="N14" s="22" t="s">
+      <c r="N14" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="O14" s="22"/>
-      <c r="P14" s="22" t="s">
+      <c r="O14" s="20"/>
+      <c r="P14" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="Q14" s="23" t="s">
+      <c r="Q14" s="21" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="39.5" customHeight="1">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="H15" s="25" t="s">
+      <c r="H15" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="I15" s="25" t="s">
+      <c r="I15" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25" t="s">
+      <c r="J15" s="23"/>
+      <c r="K15" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="L15" s="25" t="s">
+      <c r="L15" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="M15" s="25" t="s">
+      <c r="M15" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="N15" s="25" t="s">
+      <c r="N15" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="O15" s="25" t="s">
+      <c r="O15" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="P15" s="25" t="s">
+      <c r="P15" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q15" s="26" t="s">
+      <c r="Q15" s="24" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="39.5" customHeight="1">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="25" t="s">
+      <c r="F16" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="H16" s="25" t="s">
+      <c r="H16" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="I16" s="25" t="s">
+      <c r="I16" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25" t="s">
+      <c r="J16" s="23"/>
+      <c r="K16" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="L16" s="25" t="s">
+      <c r="L16" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="M16" s="25" t="s">
+      <c r="M16" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="N16" s="25" t="s">
+      <c r="N16" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="O16" s="25" t="s">
+      <c r="O16" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="P16" s="25" t="s">
+      <c r="P16" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="Q16" s="26" t="s">
+      <c r="Q16" s="24" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="39.5" customHeight="1">
-      <c r="A17" s="27" t="s">
+      <c r="A17" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="E17" s="28" t="s">
+      <c r="E17" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="G17" s="28" t="s">
+      <c r="G17" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="H17" s="28" t="s">
+      <c r="H17" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="I17" s="25" t="s">
+      <c r="I17" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28" t="s">
+      <c r="J17" s="26"/>
+      <c r="K17" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="L17" s="28" t="s">
+      <c r="L17" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="M17" s="28" t="s">
+      <c r="M17" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="N17" s="28" t="s">
+      <c r="N17" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="O17" s="28" t="s">
+      <c r="O17" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="P17" s="28" t="s">
+      <c r="P17" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="Q17" s="29" t="s">
+      <c r="Q17" s="27" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="C18" s="31" t="s">
+      <c r="C18" s="29" t="s">
         <v>137</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="E18" s="31" t="s">
+      <c r="E18" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="H18" s="31" t="s">
+      <c r="H18" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="I18" s="31" t="s">
+      <c r="I18" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="31" t="s">
+      <c r="J18" s="29"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="M18" s="31" t="s">
+      <c r="M18" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="N18" s="31" t="s">
+      <c r="N18" s="29" t="s">
         <v>143</v>
       </c>
-      <c r="O18" s="31" t="s">
+      <c r="O18" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="P18" s="31" t="s">
+      <c r="P18" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="Q18" s="32" t="s">
+      <c r="Q18" s="30" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="32" t="s">
         <v>146</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="E19" s="34" t="s">
+      <c r="E19" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="34" t="s">
+      <c r="F19" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="H19" s="34" t="s">
+      <c r="H19" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="I19" s="31" t="s">
+      <c r="I19" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34" t="s">
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="M19" s="34" t="s">
+      <c r="M19" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="N19" s="34" t="s">
+      <c r="N19" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="O19" s="34" t="s">
+      <c r="O19" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="P19" s="34" t="s">
+      <c r="P19" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="Q19" s="35" t="s">
+      <c r="Q19" s="33" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="26.25" customHeight="1">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="C20" s="37" t="s">
+      <c r="C20" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="E20" s="37" t="s">
+      <c r="E20" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="37" t="s">
+      <c r="F20" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="G20" s="37" t="s">
+      <c r="G20" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="H20" s="37" t="s">
+      <c r="H20" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="I20" s="31" t="s">
+      <c r="I20" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="J20" s="37"/>
-      <c r="K20" s="37"/>
-      <c r="L20" s="37" t="s">
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="M20" s="37" t="s">
+      <c r="M20" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="N20" s="37" t="s">
+      <c r="N20" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="O20" s="37" t="s">
+      <c r="O20" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="P20" s="37" t="s">
+      <c r="P20" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="Q20" s="38" t="s">
+      <c r="Q20" s="36" t="s">
         <v>165</v>
       </c>
     </row>

</xml_diff>